<commit_message>
Add 60 RUB/unit fulfillment to P&L and record rule in CLAUDE.md
- Fulfillment 60 RUB/unit (packaging, warehouse, staff salaries) added to
  cost of goods sold: -184500 RUB (60 x 3075 units)
- Profit before tax revised: 911540 -> 727040 RUB
- CLAUDE.md: effective cost = last-arrival cost + 60 RUB fulfillment

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_0153XBqtvJYtRAKHdw3RmMsz
</commit_message>
<xml_diff>
--- a/outputs/ozon_pnl/ozon_pnl_nachisleniya_01-29.09.2026.xlsx
+++ b/outputs/ozon_pnl/ozon_pnl_nachisleniya_01-29.09.2026.xlsx
@@ -479,10 +479,10 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C25"/>
+  <dimension ref="A1:C26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="44" customWidth="1" min="1" max="1"/>
+    <col width="46" customWidth="1" min="1" max="1"/>
     <col width="16" customWidth="1" min="2" max="2"/>
     <col width="44" customWidth="1" min="3" max="3"/>
   </cols>
@@ -582,7 +582,7 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>РАСХОДЫ</t>
+          <t>РАСХОДЫ OZON</t>
         </is>
       </c>
       <c r="B10" s="4" t="n"/>
@@ -770,15 +770,30 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Фулфилмент 60 ₽/шт (упаковка/склад/зарплаты)</t>
+        </is>
+      </c>
+      <c r="B25" s="7" t="n">
+        <v>-184500</v>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>60 ₽ × 3 075 шт</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="8" t="inlineStr">
         <is>
           <t>ПРИБЫЛЬ до налога</t>
         </is>
       </c>
-      <c r="B25" s="9" t="n">
-        <v>911540</v>
-      </c>
-      <c r="C25" s="10" t="inlineStr">
+      <c r="B26" s="9" t="n">
+        <v>727040</v>
+      </c>
+      <c r="C26" s="10" t="inlineStr">
         <is>
           <t>До вычета УСН+НДС 5%</t>
         </is>
@@ -844,7 +859,7 @@
     <row r="7">
       <c r="A7" s="12" t="inlineStr">
         <is>
-          <t>Часть начислений (реклама, депозиты, штрафы) без привязки к схеме — не вошли в разбивку.</t>
+          <t>Реклама, депозиты, штрафы без привязки к схеме в разбивку не вошли.</t>
         </is>
       </c>
     </row>

</xml_diff>